<commit_message>
Forms sync auto batch 6: 5000 files
</commit_message>
<xml_diff>
--- a/order_forms/029_nft_marketplace_inquiry_form--order_forms.xlsx
+++ b/order_forms/029_nft_marketplace_inquiry_form--order_forms.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -814,7 +814,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>nft_marketplace_1</t>
+          <t>nft marketplace 1</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>nft_marketplace_2</t>
+          <t>nft marketplace 2</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nft_marketplace_3</t>
+          <t>nft marketplace 3</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>nft_tag_1</t>
+          <t>nft tag 1</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>nft_tag_2</t>
+          <t>nft tag 2</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>nft_tag_3</t>
+          <t>nft tag 3</t>
         </is>
       </c>
     </row>

</xml_diff>